<commit_message>
Actualización planes de inversión
</commit_message>
<xml_diff>
--- a/data/RIGI_planes_inversion.xlsx
+++ b/data/RIGI_planes_inversion.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="126">
   <si>
     <t xml:space="preserve">anio</t>
   </si>
@@ -59,7 +59,7 @@
     <t xml:space="preserve">https://www.argentina.gob.ar/economia/rigi</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-08-14T14:55:36-03:00</t>
+    <t xml:space="preserve">2026-08-29T20:09:29-03:00</t>
   </si>
   <si>
     <t xml:space="preserve">petroleo</t>
@@ -206,6 +206,9 @@
     <t xml:space="preserve">Sin diferencias.</t>
   </si>
   <si>
+    <t xml:space="preserve">Minería: publicado=1473, calculado=1472, diferencia=1; Total desde subsectores: gráfico=3701, suma_subsectores=3700, diferencia=1</t>
+  </si>
+  <si>
     <t xml:space="preserve">campo</t>
   </si>
   <si>
@@ -254,13 +257,13 @@
     <t xml:space="preserve">last_modified</t>
   </si>
   <si>
-    <t xml:space="preserve">Fri, 14 Aug 2026 16:09:19 GMT</t>
+    <t xml:space="preserve">Sat, 29 Aug 2026 20:19:23 GMT</t>
   </si>
   <si>
     <t xml:space="preserve">html_bytes</t>
   </si>
   <si>
-    <t xml:space="preserve">84137</t>
+    <t xml:space="preserve">76172</t>
   </si>
   <si>
     <t xml:space="preserve">cantidad_intentos</t>
@@ -350,9 +353,6 @@
     <t xml:space="preserve">inconsistencias_detectadas</t>
   </si>
   <si>
-    <t xml:space="preserve">Ninguna.</t>
-  </si>
-  <si>
     <t xml:space="preserve">cambios_referencia_2026</t>
   </si>
   <si>
@@ -362,16 +362,19 @@
     <t xml:space="preserve">advertencias_ejecucion</t>
   </si>
   <si>
+    <t xml:space="preserve">Ninguna.</t>
+  </si>
+  <si>
     <t xml:space="preserve">sha256_json_embebido</t>
   </si>
   <si>
-    <t xml:space="preserve">4d4cb72b3585bc2d72f993c99e8f3bf6165bb14dd24a50dad49c38bc8a13dafd</t>
+    <t xml:space="preserve">25cfef15cc20c42d34f5a7875a7eb674a699182e4fc9c32e6edef676e26e8b95</t>
   </si>
   <si>
     <t xml:space="preserve">sha256_html</t>
   </si>
   <si>
-    <t xml:space="preserve">d4e5a6e1039fae4c4e5a761563ca4e27d4683a62fbb81886ea4c78c1994caa85</t>
+    <t xml:space="preserve">22ade973790c5a71728f7f00feae76c55f901530af940249554cb88a7ae4c78c</t>
   </si>
   <si>
     <t xml:space="preserve">version_R</t>
@@ -399,7 +402,7 @@
   <numFmts count="1">
     <numFmt numFmtId="166" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -424,8 +427,14 @@
       <name val="Calibri"/>
       <b/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF991B1B"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -440,6 +449,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -460,13 +474,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -914,7 +929,7 @@
         <v>37</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H2" t="s">
         <v>13</v>
@@ -943,13 +958,13 @@
         <v>17</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H3" t="s">
         <v>13</v>
@@ -981,10 +996,10 @@
         <v>14</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H4" t="s">
         <v>13</v>
@@ -1019,7 +1034,7 @@
         <v>527</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H5" t="s">
         <v>13</v>
@@ -1054,7 +1069,7 @@
         <v>527</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H6" t="s">
         <v>13</v>
@@ -1089,7 +1104,7 @@
         <v>527</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H7" t="s">
         <v>13</v>
@@ -1124,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H8" t="s">
         <v>13</v>
@@ -1159,7 +1174,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H9" t="s">
         <v>13</v>
@@ -1194,7 +1209,7 @@
         <v>252</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H10" t="s">
         <v>13</v>
@@ -1223,13 +1238,13 @@
         <v>17</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1565</v>
+        <v>1574</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1793</v>
+        <v>1802</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H11" t="s">
         <v>13</v>
@@ -1261,10 +1276,10 @@
         <v>228</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1793</v>
+        <v>1802</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H12" t="s">
         <v>13</v>
@@ -1296,10 +1311,10 @@
         <v>419</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H13" t="s">
         <v>13</v>
@@ -1331,10 +1346,10 @@
         <v>948</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H14" t="s">
         <v>13</v>
@@ -1366,10 +1381,10 @@
         <v>105</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H15" t="s">
         <v>13</v>
@@ -1404,7 +1419,7 @@
         <v>82</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H16" t="s">
         <v>13</v>
@@ -1439,7 +1454,7 @@
         <v>92</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="H17" t="s">
         <v>13</v>
@@ -1474,7 +1489,7 @@
         <v>162</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H18" t="s">
         <v>13</v>
@@ -1503,13 +1518,13 @@
         <v>17</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2277</v>
+        <v>2348</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>2653</v>
+        <v>2724</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H19" t="s">
         <v>13</v>
@@ -1541,10 +1556,10 @@
         <v>376</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>2653</v>
+        <v>2724</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H20" t="s">
         <v>13</v>
@@ -1579,7 +1594,7 @@
         <v>2579</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H21" t="s">
         <v>13</v>
@@ -1614,7 +1629,7 @@
         <v>2579</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H22" t="s">
         <v>13</v>
@@ -1649,7 +1664,7 @@
         <v>2579</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H23" t="s">
         <v>13</v>
@@ -1684,7 +1699,7 @@
         <v>130</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H24" t="s">
         <v>13</v>
@@ -1719,7 +1734,7 @@
         <v>74</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="H25" t="s">
         <v>13</v>
@@ -1754,7 +1769,7 @@
         <v>36</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H26" t="s">
         <v>13</v>
@@ -1783,13 +1798,13 @@
         <v>17</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>959</v>
+        <v>1090</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>1501</v>
+        <v>1632</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H27" t="s">
         <v>13</v>
@@ -1821,10 +1836,10 @@
         <v>542</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1501</v>
+        <v>1632</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H28" t="s">
         <v>13</v>
@@ -1859,7 +1874,7 @@
         <v>3875</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H29" t="s">
         <v>13</v>
@@ -1894,7 +1909,7 @@
         <v>3875</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H30" t="s">
         <v>13</v>
@@ -1929,7 +1944,7 @@
         <v>3875</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H31" t="s">
         <v>13</v>
@@ -1964,7 +1979,7 @@
         <v>66</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H32" t="s">
         <v>13</v>
@@ -1999,7 +2014,7 @@
         <v>64</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="H33" t="s">
         <v>13</v>
@@ -2034,7 +2049,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H34" t="s">
         <v>13</v>
@@ -2063,13 +2078,13 @@
         <v>17</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>680</v>
+        <v>818</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>1171</v>
+        <v>1309</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H35" t="s">
         <v>13</v>
@@ -2101,10 +2116,10 @@
         <v>491</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>1171</v>
+        <v>1309</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H36" t="s">
         <v>13</v>
@@ -2139,7 +2154,7 @@
         <v>4128</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H37" t="s">
         <v>13</v>
@@ -2174,7 +2189,7 @@
         <v>4128</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H38" t="s">
         <v>13</v>
@@ -2209,7 +2224,7 @@
         <v>4128</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H39" t="s">
         <v>13</v>
@@ -2244,7 +2259,7 @@
         <v>8</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H40" t="s">
         <v>13</v>
@@ -2279,7 +2294,7 @@
         <v>24</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="H41" t="s">
         <v>13</v>
@@ -10212,7 +10227,7 @@
         <v>37</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>527</v>
@@ -10224,7 +10239,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>14</v>
@@ -10242,7 +10257,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
     </row>
     <row r="3">
@@ -10253,10 +10268,10 @@
         <v>252</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1793</v>
+        <v>1802</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>82</v>
@@ -10265,7 +10280,7 @@
         <v>92</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1565</v>
+        <v>1574</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>228</v>
@@ -10283,7 +10298,7 @@
         <v>92</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
     </row>
     <row r="4">
@@ -10294,7 +10309,7 @@
         <v>162</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2653</v>
+        <v>2724</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>2579</v>
@@ -10306,7 +10321,7 @@
         <v>74</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2277</v>
+        <v>2348</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>376</v>
@@ -10324,7 +10339,7 @@
         <v>74</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
     </row>
     <row r="5">
@@ -10335,7 +10350,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1501</v>
+        <v>1632</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>3875</v>
@@ -10347,7 +10362,7 @@
         <v>64</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>959</v>
+        <v>1090</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>542</v>
@@ -10365,7 +10380,7 @@
         <v>64</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
     </row>
     <row r="6">
@@ -10376,7 +10391,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1171</v>
+        <v>1309</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>4128</v>
@@ -10388,7 +10403,7 @@
         <v>24</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>680</v>
+        <v>818</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>491</v>
@@ -10406,7 +10421,7 @@
         <v>24</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
     </row>
     <row r="7">
@@ -11676,10 +11691,10 @@
         <v>2024</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0</v>
@@ -11712,10 +11727,10 @@
         <v>1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>0</v>
@@ -11724,7 +11739,7 @@
         <v>1</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>0</v>
@@ -11741,7 +11756,7 @@
       <c r="W2" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="X2" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -11750,10 +11765,10 @@
         <v>2025</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1793</v>
+        <v>1802</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1793</v>
+        <v>1802</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>0</v>
@@ -11762,16 +11777,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>1472</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3" t="b">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="I3" s="4" t="b">
+        <v>0</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>92</v>
@@ -11786,10 +11801,10 @@
         <v>1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>3691</v>
+        <v>3701</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>0</v>
@@ -11798,13 +11813,13 @@
         <v>1</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>3691</v>
+        <v>3700</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="3" t="b">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="T3" s="4" t="b">
+        <v>0</v>
       </c>
       <c r="U3" s="2" t="n">
         <v>0</v>
@@ -11812,11 +11827,11 @@
       <c r="V3" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="W3" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>62</v>
+      <c r="W3" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="4">
@@ -11824,10 +11839,10 @@
         <v>2026</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>2653</v>
+        <v>2724</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2653</v>
+        <v>2724</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -11860,10 +11875,10 @@
         <v>1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="P4" s="2" t="n">
         <v>0</v>
@@ -11872,7 +11887,7 @@
         <v>1</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>5598</v>
+        <v>5669</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>0</v>
@@ -11889,7 +11904,7 @@
       <c r="W4" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X4" s="4" t="s">
+      <c r="X4" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -11898,10 +11913,10 @@
         <v>2027</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1501</v>
+        <v>1632</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1501</v>
+        <v>1632</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0</v>
@@ -11934,10 +11949,10 @@
         <v>1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="P5" s="2" t="n">
         <v>0</v>
@@ -11946,7 +11961,7 @@
         <v>1</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>5542</v>
+        <v>5673</v>
       </c>
       <c r="S5" s="2" t="n">
         <v>0</v>
@@ -11963,7 +11978,7 @@
       <c r="W5" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X5" s="4" t="s">
+      <c r="X5" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -11972,10 +11987,10 @@
         <v>2028</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1171</v>
+        <v>1309</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1171</v>
+        <v>1309</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>0</v>
@@ -12008,10 +12023,10 @@
         <v>1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="P6" s="2" t="n">
         <v>0</v>
@@ -12020,7 +12035,7 @@
         <v>1</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>5331</v>
+        <v>5469</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>0</v>
@@ -12037,7 +12052,7 @@
       <c r="W6" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X6" s="4" t="s">
+      <c r="X6" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12111,7 +12126,7 @@
       <c r="W7" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X7" s="4" t="s">
+      <c r="X7" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12185,7 +12200,7 @@
       <c r="W8" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X8" s="4" t="s">
+      <c r="X8" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12259,7 +12274,7 @@
       <c r="W9" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X9" s="4" t="s">
+      <c r="X9" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12333,7 +12348,7 @@
       <c r="W10" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X10" s="4" t="s">
+      <c r="X10" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12407,7 +12422,7 @@
       <c r="W11" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X11" s="4" t="s">
+      <c r="X11" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12481,7 +12496,7 @@
       <c r="W12" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X12" s="4" t="s">
+      <c r="X12" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12555,7 +12570,7 @@
       <c r="W13" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X13" s="4" t="s">
+      <c r="X13" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12629,7 +12644,7 @@
       <c r="W14" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X14" s="4" t="s">
+      <c r="X14" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12703,7 +12718,7 @@
       <c r="W15" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X15" s="4" t="s">
+      <c r="X15" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12777,7 +12792,7 @@
       <c r="W16" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X16" s="4" t="s">
+      <c r="X16" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12851,7 +12866,7 @@
       <c r="W17" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X17" s="4" t="s">
+      <c r="X17" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12925,7 +12940,7 @@
       <c r="W18" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X18" s="4" t="s">
+      <c r="X18" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12999,7 +13014,7 @@
       <c r="W19" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X19" s="4" t="s">
+      <c r="X19" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13073,7 +13088,7 @@
       <c r="W20" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X20" s="4" t="s">
+      <c r="X20" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13147,7 +13162,7 @@
       <c r="W21" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X21" s="4" t="s">
+      <c r="X21" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13221,7 +13236,7 @@
       <c r="W22" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X22" s="4" t="s">
+      <c r="X22" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13295,7 +13310,7 @@
       <c r="W23" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X23" s="4" t="s">
+      <c r="X23" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13369,7 +13384,7 @@
       <c r="W24" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X24" s="4" t="s">
+      <c r="X24" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13443,7 +13458,7 @@
       <c r="W25" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X25" s="4" t="s">
+      <c r="X25" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13517,7 +13532,7 @@
       <c r="W26" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X26" s="4" t="s">
+      <c r="X26" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13591,7 +13606,7 @@
       <c r="W27" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X27" s="4" t="s">
+      <c r="X27" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13665,7 +13680,7 @@
       <c r="W28" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X28" s="4" t="s">
+      <c r="X28" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13739,7 +13754,7 @@
       <c r="W29" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X29" s="4" t="s">
+      <c r="X29" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13813,7 +13828,7 @@
       <c r="W30" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X30" s="4" t="s">
+      <c r="X30" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13887,7 +13902,7 @@
       <c r="W31" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X31" s="4" t="s">
+      <c r="X31" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -13961,7 +13976,7 @@
       <c r="W32" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X32" s="4" t="s">
+      <c r="X32" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -14035,7 +14050,7 @@
       <c r="W33" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X33" s="4" t="s">
+      <c r="X33" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -14109,7 +14124,7 @@
       <c r="W34" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="X34" s="4" t="s">
+      <c r="X34" s="5" t="s">
         <v>62</v>
       </c>
     </row>
@@ -14133,225 +14148,225 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="4" t="s">
         <v>69</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="4" t="s">
         <v>71</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B7" s="4" t="s">
         <v>73</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="4" t="s">
         <v>75</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="4" t="s">
         <v>77</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="4" t="s">
         <v>79</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>80</v>
-      </c>
-      <c r="B11" s="4" t="s">
         <v>81</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>82</v>
-      </c>
-      <c r="B12" s="4" t="s">
         <v>83</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B13" s="4" t="s">
         <v>85</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B14" s="4" t="s">
         <v>87</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>88</v>
-      </c>
-      <c r="B15" s="4" t="s">
         <v>89</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>90</v>
-      </c>
-      <c r="B16" s="4" t="s">
         <v>91</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>92</v>
-      </c>
-      <c r="B17" s="4" t="s">
         <v>93</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>94</v>
-      </c>
-      <c r="B18" s="4" t="s">
         <v>95</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>96</v>
-      </c>
-      <c r="B19" s="4" t="s">
         <v>97</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>98</v>
-      </c>
-      <c r="B20" s="4" t="s">
         <v>99</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>100</v>
-      </c>
-      <c r="B21" s="4" t="s">
         <v>101</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>102</v>
-      </c>
-      <c r="B22" s="4" t="s">
         <v>103</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>104</v>
-      </c>
-      <c r="B23" s="4" t="s">
         <v>105</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>106</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>93</v>
+        <v>107</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>107</v>
-      </c>
-      <c r="B25" s="4" t="s">
         <v>108</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>109</v>
+      <c r="B26" s="5" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>110</v>
-      </c>
-      <c r="B27" s="4" t="s">
         <v>111</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
         <v>112</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>113</v>
       </c>
     </row>
@@ -14359,48 +14374,48 @@
       <c r="A29" t="s">
         <v>114</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>111</v>
+      <c r="B29" s="5" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30" s="4" t="s">
         <v>116</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>117</v>
-      </c>
-      <c r="B31" s="4" t="s">
         <v>118</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>119</v>
-      </c>
-      <c r="B32" s="4" t="s">
         <v>120</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>121</v>
-      </c>
-      <c r="B33" s="4" t="s">
         <v>122</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>123</v>
-      </c>
-      <c r="B34" s="4" t="s">
         <v>124</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>